<commit_message>
chore (flashcards) : maj des documents
</commit_message>
<xml_diff>
--- a/Doc_readme/Journal-de-Travail_DamienChabal.xlsx
+++ b/Doc_readme/Journal-de-Travail_DamienChabal.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\damie\Documents\P_AppMobile\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pv77ngi\Documents\GitHub\P_AppMobile\Doc_readme\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26C0C940-B2D2-46D5-96D5-2C3DE7D57112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5A06131-C759-463B-8B5D-685593EB1620}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2400" yWindow="795" windowWidth="15060" windowHeight="14295" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="4575" yWindow="1950" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="49">
   <si>
     <t>Auteur:</t>
   </si>
@@ -185,6 +185,9 @@
   </si>
   <si>
     <t>Ajout de la gestion des tages et filtrage</t>
+  </si>
+  <si>
+    <t>Completion des documents a rendre</t>
   </si>
 </sst>
 </file>
@@ -1133,7 +1136,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>60</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1197,7 +1200,6 @@
     </c:legend>
     <c:plotVisOnly val="0"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1205,6 +1207,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1544,7 +1547,6 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1552,6 +1554,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1979,13 +1982,13 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1</c:v>
+                  <c:v>0.94594594594594594</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>5.4054054054054057E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2140,7 +2143,6 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2148,6 +2150,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -4220,7 +4223,7 @@
       <c r="B3" s="82"/>
       <c r="C3" s="78" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>17 heures 30 minutes</v>
+        <v>18 heures 30 minutes</v>
       </c>
       <c r="D3" s="19"/>
       <c r="E3" s="3"/>
@@ -4233,7 +4236,7 @@
       <c r="B4" s="5"/>
       <c r="C4" s="19">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>780</v>
+        <v>840</v>
       </c>
       <c r="D4" s="19">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
@@ -4241,7 +4244,7 @@
       </c>
       <c r="E4" s="29">
         <f>SUM(C4:D4)</f>
-        <v>1050</v>
+        <v>1110</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4701,7 +4704,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="36">
-        <v>46167</v>
+        <v>46169</v>
       </c>
       <c r="C24" s="37">
         <v>1</v>
@@ -4721,10 +4724,16 @@
         <v/>
       </c>
       <c r="B25" s="40"/>
-      <c r="C25" s="41"/>
+      <c r="C25" s="41">
+        <v>1</v>
+      </c>
       <c r="D25" s="42"/>
-      <c r="E25" s="43"/>
-      <c r="F25" s="28"/>
+      <c r="E25" s="43" t="s">
+        <v>4</v>
+      </c>
+      <c r="F25" s="28" t="s">
+        <v>48</v>
+      </c>
       <c r="G25" s="46"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
@@ -10999,7 +11008,7 @@
       </c>
       <c r="G7" s="56">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$10</f>
-        <v>1</v>
+        <v>0.94594594594594594</v>
       </c>
       <c r="L7" s="64" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11053,7 +11062,7 @@
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="B9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$D$7:$D$532)</f>
@@ -11061,7 +11070,7 @@
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="E9" s="23" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11069,11 +11078,11 @@
       </c>
       <c r="F9" s="55" t="str">
         <f t="shared" si="1"/>
-        <v>0 h 00 min</v>
+        <v>1 h 00 min</v>
       </c>
       <c r="G9" s="56">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>5.4054054054054057E-2</v>
       </c>
       <c r="L9" s="66" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11090,7 +11099,7 @@
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10">
         <f>SUM(A6:A9)</f>
-        <v>780</v>
+        <v>840</v>
       </c>
       <c r="B10">
         <f>SUM(B6:B9)</f>
@@ -11098,18 +11107,18 @@
       </c>
       <c r="C10">
         <f>SUM(A10:B10)</f>
-        <v>1050</v>
+        <v>1110</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>18</v>
       </c>
       <c r="F10" s="50" t="str">
         <f t="shared" si="1"/>
-        <v>17 h 30 min</v>
+        <v>18 h 30 min</v>
       </c>
       <c r="G10" s="57">
         <f>C10/C11</f>
-        <v>0.19886363636363635</v>
+        <v>0.21022727272727273</v>
       </c>
       <c r="L10" s="67" t="s">
         <v>18</v>
@@ -11148,15 +11157,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="eefa3612-053e-497a-ae76-8a76877f5e22" xsi:nil="true"/>
@@ -11166,6 +11166,15 @@
     <img xmlns="b5cf4370-ac38-4b9e-9836-ef6f5df64f24" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11382,14 +11391,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -11398,6 +11399,14 @@
     <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
     <ds:schemaRef ds:uri="eefa3612-053e-497a-ae76-8a76877f5e22"/>
     <ds:schemaRef ds:uri="b5cf4370-ac38-4b9e-9836-ef6f5df64f24"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>